<commit_message>
finalise entry of 2024 data
</commit_message>
<xml_diff>
--- a/dat/invasion-front-reconnaissance-data.xlsx
+++ b/dat/invasion-front-reconnaissance-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/293003c_curtin_edu_au/Documents/Projects/TCZ-research/invasion-front-monitoring/dat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="314" documentId="8_{B727244B-ED70-C849-9045-E4097DDF71FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66187FB8-315F-FC43-B045-62001FDD1C37}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="8_{B727244B-ED70-C849-9045-E4097DDF71FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{032E5FCD-E1FC-0949-B772-4E5DD5B3A87F}"/>
   <bookViews>
-    <workbookView xWindow="520" yWindow="1380" windowWidth="20240" windowHeight="15520" xr2:uid="{4CAA4207-9EE1-5144-A1AD-9EE0DFB21093}"/>
+    <workbookView xWindow="9640" yWindow="1220" windowWidth="20240" windowHeight="15520" xr2:uid="{4CAA4207-9EE1-5144-A1AD-9EE0DFB21093}"/>
   </bookViews>
   <sheets>
     <sheet name="recon_data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="47">
   <si>
     <t>A place where all Tim and Ben's surveys go</t>
   </si>
@@ -157,16 +157,50 @@
   </si>
   <si>
     <t>12+ freshwater crocs in the lagoon.</t>
+  </si>
+  <si>
+    <t>2024-10-26-1</t>
+  </si>
+  <si>
+    <t>2024-10-26-2</t>
+  </si>
+  <si>
+    <t>2024-10-26-3</t>
+  </si>
+  <si>
+    <t>2024-10-26-4</t>
+  </si>
+  <si>
+    <t>2024-10-26-5</t>
+  </si>
+  <si>
+    <t>2024-10-26-6</t>
+  </si>
+  <si>
+    <t>2024-10-26-7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -192,10 +226,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813D5425-8307-4A4E-BBA1-7FF7DA274487}">
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
@@ -1641,7 +1678,7 @@
         <v>10</v>
       </c>
       <c r="G29">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H29" s="2">
         <v>0.77083333333333337</v>
@@ -1685,7 +1722,7 @@
         <v>10</v>
       </c>
       <c r="G30">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H30" s="1">
         <v>0.81944444444444442</v>
@@ -1726,7 +1763,7 @@
         <v>10</v>
       </c>
       <c r="G31">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H31" s="1">
         <v>0.84375</v>
@@ -1767,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="G32">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H32" s="1">
         <v>0.85416666666666663</v>
@@ -1808,7 +1845,7 @@
         <v>10</v>
       </c>
       <c r="G33">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H33" s="2">
         <v>0.86805555555555558</v>
@@ -1852,7 +1889,7 @@
         <v>10</v>
       </c>
       <c r="G34">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H34" s="1">
         <v>0.87847222222222221</v>
@@ -1896,7 +1933,7 @@
         <v>10</v>
       </c>
       <c r="G35">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H35" s="2">
         <v>0.89236111111111116</v>
@@ -1940,7 +1977,7 @@
         <v>10</v>
       </c>
       <c r="G36">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H36" s="2">
         <v>0.90625</v>
@@ -1984,7 +2021,7 @@
         <v>10</v>
       </c>
       <c r="G37">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H37" s="2">
         <v>0.92361111111111116</v>
@@ -2028,7 +2065,7 @@
         <v>10</v>
       </c>
       <c r="G38">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H38" s="2">
         <v>0.93402777777777779</v>
@@ -2052,7 +2089,336 @@
         <v>39</v>
       </c>
     </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39">
+        <v>-18.315550000000002</v>
+      </c>
+      <c r="C39">
+        <v>123.72669999999999</v>
+      </c>
+      <c r="D39">
+        <v>56</v>
+      </c>
+      <c r="E39">
+        <v>2024</v>
+      </c>
+      <c r="F39">
+        <v>10</v>
+      </c>
+      <c r="G39">
+        <v>26</v>
+      </c>
+      <c r="H39" s="2">
+        <v>0.77222222222222225</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>16</v>
+      </c>
+      <c r="K39">
+        <v>38</v>
+      </c>
+      <c r="L39" t="s">
+        <v>19</v>
+      </c>
+      <c r="M39" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>79</v>
+      </c>
+      <c r="B40">
+        <v>-18.270114979999999</v>
+      </c>
+      <c r="C40">
+        <v>123.748251</v>
+      </c>
+      <c r="D40">
+        <v>62.396934999999999</v>
+      </c>
+      <c r="E40">
+        <v>2024</v>
+      </c>
+      <c r="F40">
+        <v>10</v>
+      </c>
+      <c r="G40">
+        <v>26</v>
+      </c>
+      <c r="H40" s="2">
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>20</v>
+      </c>
+      <c r="K40">
+        <v>34</v>
+      </c>
+      <c r="L40" t="s">
+        <v>19</v>
+      </c>
+      <c r="M40" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41">
+        <v>-18.25459</v>
+      </c>
+      <c r="C41">
+        <v>123.66200000000001</v>
+      </c>
+      <c r="D41">
+        <v>90</v>
+      </c>
+      <c r="E41">
+        <v>2024</v>
+      </c>
+      <c r="F41">
+        <v>10</v>
+      </c>
+      <c r="G41">
+        <v>26</v>
+      </c>
+      <c r="H41" s="2">
+        <v>0.81111111111111112</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>6</v>
+      </c>
+      <c r="K41">
+        <v>35</v>
+      </c>
+      <c r="L41" t="s">
+        <v>19</v>
+      </c>
+      <c r="M41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42">
+        <v>-18.196650000000002</v>
+      </c>
+      <c r="C42">
+        <v>123.64870000000001</v>
+      </c>
+      <c r="D42">
+        <v>69</v>
+      </c>
+      <c r="E42">
+        <v>2024</v>
+      </c>
+      <c r="F42">
+        <v>10</v>
+      </c>
+      <c r="G42">
+        <v>26</v>
+      </c>
+      <c r="H42" s="2">
+        <v>0.82638888888888884</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>4</v>
+      </c>
+      <c r="K42">
+        <v>34</v>
+      </c>
+      <c r="L42" t="s">
+        <v>19</v>
+      </c>
+      <c r="M42" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43">
+        <v>-18.14696</v>
+      </c>
+      <c r="C43">
+        <v>123.6169</v>
+      </c>
+      <c r="D43">
+        <v>114</v>
+      </c>
+      <c r="E43">
+        <v>2024</v>
+      </c>
+      <c r="F43">
+        <v>10</v>
+      </c>
+      <c r="G43">
+        <v>26</v>
+      </c>
+      <c r="H43" s="2">
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>10</v>
+      </c>
+      <c r="K43">
+        <v>32</v>
+      </c>
+      <c r="L43" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44">
+        <v>-18.062999999999999</v>
+      </c>
+      <c r="C44">
+        <v>123.54730000000001</v>
+      </c>
+      <c r="D44">
+        <v>61</v>
+      </c>
+      <c r="E44">
+        <v>2024</v>
+      </c>
+      <c r="F44">
+        <v>10</v>
+      </c>
+      <c r="G44">
+        <v>26</v>
+      </c>
+      <c r="H44" s="2">
+        <v>0.8520833333333333</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>6</v>
+      </c>
+      <c r="K44">
+        <v>32</v>
+      </c>
+      <c r="L44" t="s">
+        <v>19</v>
+      </c>
+      <c r="M44" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>45</v>
+      </c>
+      <c r="B45">
+        <v>-17.89039</v>
+      </c>
+      <c r="C45">
+        <v>123.5878</v>
+      </c>
+      <c r="D45">
+        <v>52</v>
+      </c>
+      <c r="E45">
+        <v>2024</v>
+      </c>
+      <c r="F45">
+        <v>10</v>
+      </c>
+      <c r="G45">
+        <v>26</v>
+      </c>
+      <c r="H45" s="2">
+        <v>0.8979166666666667</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>10</v>
+      </c>
+      <c r="K45">
+        <v>33</v>
+      </c>
+      <c r="L45" t="s">
+        <v>19</v>
+      </c>
+      <c r="M45" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46">
+        <v>-17.918399999999998</v>
+      </c>
+      <c r="C46">
+        <v>123.6238</v>
+      </c>
+      <c r="D46">
+        <v>24</v>
+      </c>
+      <c r="E46">
+        <v>2024</v>
+      </c>
+      <c r="F46">
+        <v>10</v>
+      </c>
+      <c r="G46">
+        <v>26</v>
+      </c>
+      <c r="H46" s="2">
+        <v>0.91874999999999996</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46">
+        <v>20</v>
+      </c>
+      <c r="K46">
+        <v>31</v>
+      </c>
+      <c r="L46" t="s">
+        <v>19</v>
+      </c>
+      <c r="M46" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add 30s to 0 time observation
</commit_message>
<xml_diff>
--- a/dat/invasion-front-reconnaissance-data.xlsx
+++ b/dat/invasion-front-reconnaissance-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/293003c_curtin_edu_au/Documents/Projects/TCZ-research/invasion-front-monitoring/dat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="387" documentId="8_{B727244B-ED70-C849-9045-E4097DDF71FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{032E5FCD-E1FC-0949-B772-4E5DD5B3A87F}"/>
+  <xr:revisionPtr revIDLastSave="388" documentId="8_{B727244B-ED70-C849-9045-E4097DDF71FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CB18D77-21A9-2D48-9ED9-55F15C04B645}"/>
   <bookViews>
     <workbookView xWindow="9640" yWindow="1220" windowWidth="20240" windowHeight="15520" xr2:uid="{4CAA4207-9EE1-5144-A1AD-9EE0DFB21093}"/>
   </bookViews>
@@ -1898,7 +1898,7 @@
         <v>1</v>
       </c>
       <c r="J34">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K34">
         <v>31</v>

</xml_diff>

<commit_message>
merge fulcrum and earlier data
</commit_message>
<xml_diff>
--- a/dat/invasion-front-reconnaissance-data.xlsx
+++ b/dat/invasion-front-reconnaissance-data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/293003c/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/293003c_curtin_edu_au/Documents/Projects/TCZ-research/invasion-front-monitoring/dat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCF0764-FA22-154A-BAE1-F3B173D114F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{3DCF0764-FA22-154A-BAE1-F3B173D114F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD6E1E5-98FA-034F-B048-0B0A514D6509}"/>
   <bookViews>
     <workbookView xWindow="-14400" yWindow="-21100" windowWidth="26200" windowHeight="16740" xr2:uid="{4CAA4207-9EE1-5144-A1AD-9EE0DFB21093}"/>
   </bookViews>
@@ -54,12 +54,6 @@
     <t>temperature</t>
   </si>
   <si>
-    <t>survey.type</t>
-  </si>
-  <si>
-    <t>water.status</t>
-  </si>
-  <si>
     <t>NEG1</t>
   </si>
   <si>
@@ -159,9 +153,6 @@
     <t>All Lat/long data come from Ben's GPS and are recorded with the GRS 80 spheroid and GDA94 Datum</t>
   </si>
   <si>
-    <t>n.persons</t>
-  </si>
-  <si>
     <t>X_record_id</t>
   </si>
   <si>
@@ -171,9 +162,6 @@
     <t>X_longitude</t>
   </si>
   <si>
-    <t>X_date</t>
-  </si>
-  <si>
     <t>location_n</t>
   </si>
   <si>
@@ -183,9 +171,6 @@
     <t>notes</t>
   </si>
   <si>
-    <t>search.tim</t>
-  </si>
-  <si>
     <t>any_cane_t</t>
   </si>
   <si>
@@ -193,6 +178,21 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>how_many_p</t>
+  </si>
+  <si>
+    <t>search_tim</t>
+  </si>
+  <si>
+    <t>survey_type</t>
+  </si>
+  <si>
+    <t>water_available</t>
   </si>
 </sst>
 </file>
@@ -597,19 +597,19 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
         <v>41</v>
-      </c>
-      <c r="B1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E1" t="s">
-        <v>45</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
@@ -624,30 +624,30 @@
         <v>3</v>
       </c>
       <c r="J1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" t="s">
         <v>49</v>
-      </c>
-      <c r="K1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L1" t="s">
-        <v>48</v>
       </c>
       <c r="M1" t="s">
         <v>4</v>
       </c>
       <c r="N1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="O1" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>-17.732258980000001</v>
@@ -672,7 +672,7 @@
         <v>0.796875</v>
       </c>
       <c r="J2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K2">
         <v>2</v>
@@ -681,15 +681,15 @@
         <v>60</v>
       </c>
       <c r="N2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="4">
         <v>-17.83639801</v>
@@ -711,17 +711,17 @@
         <v>29</v>
       </c>
       <c r="J3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L3"/>
       <c r="N3" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -748,16 +748,16 @@
         <v>29</v>
       </c>
       <c r="J4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="N4" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" t="s">
+        <v>7</v>
+      </c>
+      <c r="P4" t="s">
         <v>11</v>
-      </c>
-      <c r="O4" t="s">
-        <v>9</v>
-      </c>
-      <c r="P4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -787,7 +787,7 @@
         <v>0.88648148148148154</v>
       </c>
       <c r="J5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K5">
         <v>2</v>
@@ -796,10 +796,10 @@
         <v>5</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -829,7 +829,7 @@
         <v>0.82465277777777779</v>
       </c>
       <c r="J6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K6">
         <v>2</v>
@@ -838,15 +838,15 @@
         <v>20</v>
       </c>
       <c r="N6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7" s="4">
         <v>-17.991384010000001</v>
@@ -859,7 +859,7 @@
         <v>2023-8-29</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F7" s="4">
         <v>2023</v>
@@ -871,17 +871,17 @@
         <v>29</v>
       </c>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L7"/>
       <c r="N7" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -911,7 +911,7 @@
         <v>0.80577546296296299</v>
       </c>
       <c r="J8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K8">
         <v>2</v>
@@ -920,10 +920,10 @@
         <v>20</v>
       </c>
       <c r="N8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -950,17 +950,17 @@
         <v>29</v>
       </c>
       <c r="J9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="L9"/>
       <c r="N9" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -990,7 +990,7 @@
         <v>0.76388888888888884</v>
       </c>
       <c r="J10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -999,10 +999,10 @@
         <v>10</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1032,7 +1032,7 @@
         <v>0.90660879629629632</v>
       </c>
       <c r="J11" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K11">
         <v>2</v>
@@ -1041,13 +1041,13 @@
         <v>5</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -1077,7 +1077,7 @@
         <v>0.86581018518518515</v>
       </c>
       <c r="J12" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K12">
         <v>2</v>
@@ -1086,10 +1086,10 @@
         <v>15</v>
       </c>
       <c r="N12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -1119,7 +1119,7 @@
         <v>0.83403935185185185</v>
       </c>
       <c r="J13" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K13">
         <v>2</v>
@@ -1128,10 +1128,10 @@
         <v>15</v>
       </c>
       <c r="N13" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O13" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -1161,7 +1161,7 @@
         <v>0.79655092592592591</v>
       </c>
       <c r="J14" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K14">
         <v>2</v>
@@ -1170,10 +1170,10 @@
         <v>30</v>
       </c>
       <c r="N14" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O14" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -1203,7 +1203,7 @@
         <v>0.92525462962962968</v>
       </c>
       <c r="J15" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -1212,13 +1212,13 @@
         <v>40</v>
       </c>
       <c r="N15" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O15" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -1248,7 +1248,7 @@
         <v>0.77144675925925921</v>
       </c>
       <c r="J16" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K16">
         <v>2</v>
@@ -1257,10 +1257,10 @@
         <v>20</v>
       </c>
       <c r="N16" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -1290,7 +1290,7 @@
         <v>0.80384259259259261</v>
       </c>
       <c r="J17" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K17">
         <v>2</v>
@@ -1299,10 +1299,10 @@
         <v>15</v>
       </c>
       <c r="N17" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -1332,7 +1332,7 @@
         <v>0.81987268518518519</v>
       </c>
       <c r="J18" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K18">
         <v>2</v>
@@ -1341,10 +1341,10 @@
         <v>15</v>
       </c>
       <c r="N18" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -1374,7 +1374,7 @@
         <v>0.83361111111111108</v>
       </c>
       <c r="J19" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K19">
         <v>2</v>
@@ -1383,10 +1383,10 @@
         <v>15</v>
       </c>
       <c r="N19" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O19" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -1416,7 +1416,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="J20" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K20">
         <v>2</v>
@@ -1425,10 +1425,10 @@
         <v>12</v>
       </c>
       <c r="N20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O20" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
@@ -1458,7 +1458,7 @@
         <v>0.7729166666666667</v>
       </c>
       <c r="J21" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K21">
         <v>2</v>
@@ -1470,10 +1470,10 @@
         <v>17</v>
       </c>
       <c r="N21" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O21" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
@@ -1503,7 +1503,7 @@
         <v>0.77847222222222223</v>
       </c>
       <c r="J22" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K22">
         <v>2</v>
@@ -1515,10 +1515,10 @@
         <v>15</v>
       </c>
       <c r="N22" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O22" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
@@ -1548,7 +1548,7 @@
         <v>0.79652777777777772</v>
       </c>
       <c r="J23" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K23">
         <v>2</v>
@@ -1560,10 +1560,10 @@
         <v>14</v>
       </c>
       <c r="N23" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O23" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
@@ -1593,7 +1593,7 @@
         <v>0.86944444444444446</v>
       </c>
       <c r="J24" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K24">
         <v>2</v>
@@ -1605,10 +1605,10 @@
         <v>15</v>
       </c>
       <c r="N24" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O24" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1638,7 +1638,7 @@
         <v>0.77777777777777779</v>
       </c>
       <c r="J25" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K25">
         <v>2</v>
@@ -1650,10 +1650,10 @@
         <v>20</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1683,7 +1683,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="J26" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K26">
         <v>2</v>
@@ -1695,10 +1695,10 @@
         <v>18</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
@@ -1728,7 +1728,7 @@
         <v>0.8125</v>
       </c>
       <c r="J27" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K27">
         <v>2</v>
@@ -1740,10 +1740,10 @@
         <v>17</v>
       </c>
       <c r="N27" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O27" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
@@ -1773,7 +1773,7 @@
         <v>0.84027777777777779</v>
       </c>
       <c r="J28" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K28">
         <v>2</v>
@@ -1785,13 +1785,13 @@
         <v>16</v>
       </c>
       <c r="N28" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O28" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P28" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
@@ -1821,7 +1821,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="J29" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K29">
         <v>2</v>
@@ -1833,13 +1833,13 @@
         <v>36</v>
       </c>
       <c r="N29" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O29" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="P29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
@@ -1869,7 +1869,7 @@
         <v>0.81944444444444442</v>
       </c>
       <c r="J30" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K30">
         <v>2</v>
@@ -1881,10 +1881,10 @@
         <v>31</v>
       </c>
       <c r="N30" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O30" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.2">
@@ -1914,7 +1914,7 @@
         <v>0.84375</v>
       </c>
       <c r="J31" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K31">
         <v>2</v>
@@ -1926,10 +1926,10 @@
         <v>31</v>
       </c>
       <c r="N31" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O31" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
@@ -1959,7 +1959,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="J32" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K32">
         <v>2</v>
@@ -1971,10 +1971,10 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.2">
@@ -2004,7 +2004,7 @@
         <v>0.86805555555555558</v>
       </c>
       <c r="J33" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K33">
         <v>2</v>
@@ -2016,13 +2016,13 @@
         <v>31</v>
       </c>
       <c r="N33" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O33" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P33" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -2052,7 +2052,7 @@
         <v>0.87847222222222221</v>
       </c>
       <c r="J34" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K34">
         <v>2</v>
@@ -2064,13 +2064,13 @@
         <v>31</v>
       </c>
       <c r="N34" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P34" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.2">
@@ -2100,7 +2100,7 @@
         <v>0.89236111111111116</v>
       </c>
       <c r="J35" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K35">
         <v>2</v>
@@ -2112,13 +2112,13 @@
         <v>30</v>
       </c>
       <c r="N35" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O35" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
@@ -2148,7 +2148,7 @@
         <v>0.90625</v>
       </c>
       <c r="J36" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K36">
         <v>2</v>
@@ -2160,13 +2160,13 @@
         <v>30</v>
       </c>
       <c r="N36" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O36" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P36" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -2196,7 +2196,7 @@
         <v>0.92361111111111116</v>
       </c>
       <c r="J37" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="K37">
         <v>2</v>
@@ -2208,13 +2208,13 @@
         <v>30</v>
       </c>
       <c r="N37" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O37" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P37" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
@@ -2244,7 +2244,7 @@
         <v>0.93402777777777779</v>
       </c>
       <c r="J38" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K38">
         <v>2</v>
@@ -2256,18 +2256,18 @@
         <v>30</v>
       </c>
       <c r="N38" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O38" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P38" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B39">
         <v>-18.315550000000002</v>
@@ -2292,7 +2292,7 @@
         <v>0.77222222222222225</v>
       </c>
       <c r="J39" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -2304,10 +2304,10 @@
         <v>38</v>
       </c>
       <c r="N39" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O39" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.2">
@@ -2337,7 +2337,7 @@
         <v>0.78749999999999998</v>
       </c>
       <c r="J40" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K40">
         <v>2</v>
@@ -2349,15 +2349,15 @@
         <v>34</v>
       </c>
       <c r="N40" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O40" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B41">
         <v>-18.25459</v>
@@ -2382,7 +2382,7 @@
         <v>0.81111111111111112</v>
       </c>
       <c r="J41" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K41">
         <v>2</v>
@@ -2394,15 +2394,15 @@
         <v>35</v>
       </c>
       <c r="N41" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O41" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B42">
         <v>-18.196650000000002</v>
@@ -2427,7 +2427,7 @@
         <v>0.82638888888888884</v>
       </c>
       <c r="J42" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K42">
         <v>2</v>
@@ -2439,15 +2439,15 @@
         <v>34</v>
       </c>
       <c r="N42" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O42" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B43">
         <v>-18.14696</v>
@@ -2472,7 +2472,7 @@
         <v>0.83750000000000002</v>
       </c>
       <c r="J43" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K43">
         <v>2</v>
@@ -2484,15 +2484,15 @@
         <v>32</v>
       </c>
       <c r="N43" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O43" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B44">
         <v>-18.062999999999999</v>
@@ -2517,7 +2517,7 @@
         <v>0.8520833333333333</v>
       </c>
       <c r="J44" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K44">
         <v>2</v>
@@ -2529,15 +2529,15 @@
         <v>32</v>
       </c>
       <c r="N44" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O44" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B45">
         <v>-17.89039</v>
@@ -2562,7 +2562,7 @@
         <v>0.8979166666666667</v>
       </c>
       <c r="J45" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K45">
         <v>2</v>
@@ -2574,15 +2574,15 @@
         <v>33</v>
       </c>
       <c r="N45" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O45" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B46">
         <v>-17.918399999999998</v>
@@ -2607,7 +2607,7 @@
         <v>0.91874999999999996</v>
       </c>
       <c r="J46" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="K46">
         <v>2</v>
@@ -2619,10 +2619,10 @@
         <v>31</v>
       </c>
       <c r="N46" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O46" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2638,12 +2638,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>